<commit_message>
Rregullim i margjinave te shablloneve.
</commit_message>
<xml_diff>
--- a/public/templates/Shablloni-1-Faqe.xlsx
+++ b/public/templates/Shablloni-1-Faqe.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\Graniti\Ferizaj\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\AAB\Viti 3 Semestri 6\Tema-Graniti\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{77EF9B25-B3D8-4977-A403-470CD5310EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA706009-BDDE-41EF-B798-3AF414EA61B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Libri ndërtimor - Construction book</t>
   </si>
@@ -163,34 +163,6 @@
     <t>Organi mbikqyrës:            ________________</t>
   </si>
   <si>
-    <t xml:space="preserve">në Gjilan dhe Ferizaj    </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Objekti-Building : </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Renovimi i zyreve regjionale  </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">  PARAMASA DHE PARALLOGARITJA E PUNIMËVE TË RENOVIMIT</t>
-  </si>
-  <si>
-    <t>TE ZYREVE ADMINISTRATIVE  TË  PENSIONEVE  NË GJILAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> - Renovimi i zyreve regjionale të pensioneve </t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">      Masa         </t>
     </r>
@@ -265,6 +237,12 @@
   <si>
     <t>71.5 x 20.00  = 1430.00</t>
   </si>
+  <si>
+    <t xml:space="preserve">Objekti-Building :  - Renovimi i zyreve regjionale të pensioneve në Gjilan dhe Ferizaj    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  PARAMASA DHE PARALLOGARITJA E PUNIMËVE TË RENOVIMIT TE ZYREVE ADMINISTRATIVE  TË  PENSIONEVE  NË GJILAN</t>
+  </si>
 </sst>
 </file>
 
@@ -273,7 +251,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -341,14 +319,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -549,9 +519,9 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -570,16 +540,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -616,7 +581,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
@@ -637,18 +602,17 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -683,6 +647,48 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1007,50 +1013,49 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="59" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="59"/>
-      <c r="H1" s="60"/>
+      <c r="F1" s="55" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="55"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="51"/>
+      <c r="G2" s="48"/>
       <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="F3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="5"/>
+      <c r="F3" s="68" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="66"/>
+      <c r="H3" s="67"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="C4" s="52"/>
-      <c r="F4" s="51" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="53"/>
-      <c r="H4" s="5"/>
+      <c r="C4" s="49"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="67"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="F5" s="51" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="53"/>
-      <c r="H5" s="5"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="67"/>
     </row>
     <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="H6" s="5"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="67"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
@@ -1073,10 +1078,13 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="5"/>
+      <c r="A9" s="72" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="73"/>
+      <c r="C9" s="73"/>
+      <c r="D9" s="73"/>
+      <c r="E9" s="74"/>
       <c r="F9" s="14" t="s">
         <v>6</v>
       </c>
@@ -1086,39 +1094,40 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="51"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="19"/>
+      <c r="A10" s="72"/>
+      <c r="B10" s="73"/>
+      <c r="C10" s="73"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="74"/>
       <c r="F10" s="4"/>
       <c r="G10" s="5"/>
       <c r="H10" s="11"/>
     </row>
-    <row r="11" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="5"/>
+    <row r="11" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="69" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="70"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="71"/>
       <c r="F11" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G11" s="5"/>
-      <c r="H11" s="11" t="s">
-        <v>31</v>
+      <c r="H11" s="78" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="6"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="8"/>
+      <c r="A12" s="75"/>
+      <c r="B12" s="76"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="77"/>
       <c r="F12" s="6"/>
       <c r="G12" s="8"/>
-      <c r="H12" s="22"/>
+      <c r="H12" s="79"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -1128,11 +1137,11 @@
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="3"/>
-      <c r="F13" s="64" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="65"/>
-      <c r="H13" s="66"/>
+      <c r="F13" s="60" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13" s="61"/>
+      <c r="H13" s="62"/>
     </row>
     <row r="14" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
@@ -1144,9 +1153,9 @@
       <c r="E14" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F14" s="67"/>
-      <c r="G14" s="68"/>
-      <c r="H14" s="69"/>
+      <c r="F14" s="63"/>
+      <c r="G14" s="64"/>
+      <c r="H14" s="65"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
@@ -1179,205 +1188,205 @@
       <c r="H16" s="9"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="62"/>
-      <c r="C17" s="62"/>
-      <c r="D17" s="62"/>
-      <c r="E17" s="63"/>
+      <c r="A17" s="57" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="58"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="59"/>
       <c r="F17" s="4"/>
       <c r="G17" s="5"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="61"/>
-      <c r="B18" s="62"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="63"/>
+      <c r="A18" s="57"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="59"/>
       <c r="F18" s="4"/>
       <c r="G18" s="5"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="2.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="61"/>
-      <c r="B19" s="62"/>
-      <c r="C19" s="62"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="63"/>
+      <c r="A19" s="57"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="58"/>
+      <c r="E19" s="59"/>
       <c r="F19" s="4"/>
       <c r="G19" s="5"/>
       <c r="H19" s="11"/>
     </row>
     <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="20"/>
-      <c r="B20" s="42"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20" s="25">
+      <c r="A20" s="18"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="22">
         <v>71.5</v>
       </c>
-      <c r="G20" s="26"/>
-      <c r="H20" s="27"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="24"/>
     </row>
     <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="56"/>
-      <c r="B21" s="57"/>
-      <c r="C21" s="57"/>
-      <c r="D21" s="58"/>
-      <c r="E21" s="40" t="s">
+      <c r="A21" s="52"/>
+      <c r="B21" s="53"/>
+      <c r="C21" s="53"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="44"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="41">
+      <c r="F21" s="41"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="38">
         <f>F20</f>
         <v>71.5</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="11.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="20"/>
-      <c r="B22" s="42"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="29"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="39"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="39"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="26"/>
     </row>
     <row r="23" spans="1:8" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="23"/>
-      <c r="B23" s="34"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="30"/>
+      <c r="A23" s="20"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="27"/>
     </row>
     <row r="24" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="23"/>
-      <c r="B24" s="34"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="32"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="29"/>
     </row>
     <row r="25" spans="1:8" ht="121.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="23"/>
-      <c r="B25" s="34"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="35"/>
-      <c r="G25" s="35"/>
-      <c r="H25" s="32"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="29"/>
     </row>
     <row r="26" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="23"/>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="33"/>
+      <c r="A26" s="20"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="35"/>
+      <c r="H26" s="30"/>
     </row>
     <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="23"/>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="47"/>
+      <c r="A27" s="20"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="44"/>
     </row>
     <row r="28" spans="1:8" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="23"/>
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="32"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="29"/>
     </row>
     <row r="29" spans="1:8" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="23"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="34"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="35"/>
-      <c r="H29" s="32"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="29"/>
     </row>
     <row r="30" spans="1:8" ht="73.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="23"/>
-      <c r="B30" s="34"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="34"/>
-      <c r="E30" s="34"/>
-      <c r="F30" s="35"/>
-      <c r="G30" s="35"/>
-      <c r="H30" s="32"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="29"/>
     </row>
     <row r="31" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="23"/>
-      <c r="B31" s="34"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="36"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="38"/>
-      <c r="H31" s="33"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="30"/>
     </row>
     <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="23"/>
-      <c r="B32" s="34"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="H32" s="47"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="35"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="44"/>
     </row>
     <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="20"/>
-      <c r="B33" s="42"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="36"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="50"/>
-      <c r="H33" s="26"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="39"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="39"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="23"/>
     </row>
     <row r="34" spans="1:8" ht="1.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="31"/>
-      <c r="B34" s="54"/>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="29"/>
+      <c r="A34" s="28"/>
+      <c r="B34" s="50"/>
+      <c r="C34" s="50"/>
+      <c r="D34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="26"/>
     </row>
     <row r="35" spans="1:8" ht="8.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="31"/>
-      <c r="B35" s="54"/>
-      <c r="C35" s="54"/>
-      <c r="D35" s="54"/>
-      <c r="E35" s="54"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="47"/>
+      <c r="A35" s="28"/>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="47"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="44"/>
     </row>
     <row r="36" spans="1:8" ht="4.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
@@ -1397,21 +1406,21 @@
     </row>
     <row r="40" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
-      <c r="E40" s="46"/>
-      <c r="F40" s="39"/>
-      <c r="G40" s="39"/>
-      <c r="H40" s="48"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="36"/>
+      <c r="G40" s="36"/>
+      <c r="H40" s="45"/>
     </row>
     <row r="41" spans="1:8" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
-      <c r="H41" s="49"/>
+      <c r="H41" s="46"/>
     </row>
     <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="20"/>
-      <c r="B42" s="42"/>
-      <c r="C42" s="42"/>
-      <c r="D42" s="42"/>
-      <c r="H42" s="49"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="39"/>
+      <c r="C42" s="39"/>
+      <c r="D42" s="39"/>
+      <c r="H42" s="46"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
@@ -1452,10 +1461,14 @@
     <row r="48" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="49" ht="25.2" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="7">
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="A17:E19"/>
     <mergeCell ref="F13:H14"/>
+    <mergeCell ref="F3:H6"/>
+    <mergeCell ref="A9:E10"/>
+    <mergeCell ref="A11:E12"/>
+    <mergeCell ref="H11:H12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="92" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Rregullime te vogla por te nevojshme ne ui,excel,style,etj.
</commit_message>
<xml_diff>
--- a/public/templates/Shablloni-1-Faqe.xlsx
+++ b/public/templates/Shablloni-1-Faqe.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\AAB\Viti 3 Semestri 6\Tema-Graniti\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA706009-BDDE-41EF-B798-3AF414EA61B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B538B555-6146-4AC4-BE34-1BFF47F7CA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -521,7 +521,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -563,19 +563,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -648,32 +638,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -996,7 +986,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.5546875" customWidth="1"/>
@@ -1013,51 +1003,51 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="55" t="s">
+      <c r="F1" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="55"/>
-      <c r="H1" s="56"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="50"/>
     </row>
     <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="48"/>
+      <c r="G2" s="42"/>
       <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="68" t="s">
+      <c r="F3" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="66"/>
-      <c r="H3" s="67"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="62"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="C4" s="49"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="67"/>
+      <c r="C4" s="43"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="62"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
-      <c r="H5" s="67"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="61"/>
+      <c r="H5" s="62"/>
     </row>
     <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="A6" s="51" t="s">
+      <c r="A6" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="67"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F6" s="61"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="62"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="H7" s="5"/>
     </row>
@@ -1078,13 +1068,13 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="72" t="s">
+      <c r="A9" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="73"/>
-      <c r="C9" s="73"/>
-      <c r="D9" s="73"/>
-      <c r="E9" s="74"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="64"/>
+      <c r="D9" s="64"/>
+      <c r="E9" s="65"/>
       <c r="F9" s="14" t="s">
         <v>6</v>
       </c>
@@ -1094,40 +1084,40 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="72"/>
-      <c r="B10" s="73"/>
-      <c r="C10" s="73"/>
-      <c r="D10" s="73"/>
-      <c r="E10" s="74"/>
+      <c r="A10" s="63"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="65"/>
       <c r="F10" s="4"/>
       <c r="G10" s="5"/>
       <c r="H10" s="11"/>
     </row>
     <row r="11" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="69" t="s">
+      <c r="A11" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="70"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="70"/>
-      <c r="E11" s="71"/>
+      <c r="B11" s="67"/>
+      <c r="C11" s="67"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="68"/>
       <c r="F11" s="4" t="s">
         <v>25</v>
       </c>
       <c r="G11" s="5"/>
-      <c r="H11" s="78" t="s">
+      <c r="H11" s="72" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="75"/>
-      <c r="B12" s="76"/>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="77"/>
+      <c r="A12" s="69"/>
+      <c r="B12" s="70"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="71"/>
       <c r="F12" s="6"/>
       <c r="G12" s="8"/>
-      <c r="H12" s="79"/>
+      <c r="H12" s="73"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -1137,11 +1127,11 @@
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="3"/>
-      <c r="F13" s="60" t="s">
+      <c r="F13" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="61"/>
-      <c r="H13" s="62"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="56"/>
     </row>
     <row r="14" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
@@ -1153,9 +1143,9 @@
       <c r="E14" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F14" s="63"/>
-      <c r="G14" s="64"/>
-      <c r="H14" s="65"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="59"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
@@ -1188,42 +1178,42 @@
       <c r="H16" s="9"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="57" t="s">
+      <c r="A17" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="58"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="58"/>
-      <c r="E17" s="59"/>
+      <c r="B17" s="52"/>
+      <c r="C17" s="52"/>
+      <c r="D17" s="52"/>
+      <c r="E17" s="53"/>
       <c r="F17" s="4"/>
       <c r="G17" s="5"/>
       <c r="H17" s="11"/>
     </row>
-    <row r="18" spans="1:8" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="57"/>
-      <c r="B18" s="58"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="58"/>
-      <c r="E18" s="59"/>
+    <row r="18" spans="1:8" ht="259.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="51"/>
+      <c r="B18" s="52"/>
+      <c r="C18" s="52"/>
+      <c r="D18" s="52"/>
+      <c r="E18" s="53"/>
       <c r="F18" s="4"/>
       <c r="G18" s="5"/>
       <c r="H18" s="11"/>
     </row>
-    <row r="19" spans="1:8" ht="2.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="57"/>
-      <c r="B19" s="58"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="59"/>
+    <row r="19" spans="1:8" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="51"/>
+      <c r="B19" s="52"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="52"/>
+      <c r="E19" s="53"/>
       <c r="F19" s="4"/>
       <c r="G19" s="5"/>
       <c r="H19" s="11"/>
     </row>
     <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="18"/>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
       <c r="E20" s="19" t="s">
         <v>28</v>
       </c>
@@ -1234,232 +1224,132 @@
       <c r="H20" s="24"/>
     </row>
     <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="52"/>
-      <c r="B21" s="53"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="54"/>
-      <c r="E21" s="37" t="s">
+      <c r="A21" s="46"/>
+      <c r="B21" s="47"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="41"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="38">
+      <c r="F21" s="35"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="32">
         <f>F20</f>
         <v>71.5</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="11.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="18"/>
-      <c r="B22" s="39"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
       <c r="H22" s="26"/>
     </row>
     <row r="23" spans="1:8" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="20"/>
-      <c r="B23" s="31"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
       <c r="E23" s="21"/>
       <c r="F23" s="25"/>
       <c r="G23" s="26"/>
       <c r="H23" s="27"/>
     </row>
-    <row r="24" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="20"/>
-      <c r="B24" s="31"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="29"/>
-    </row>
-    <row r="25" spans="1:8" ht="121.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="20"/>
-      <c r="B25" s="31"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
-      <c r="H25" s="29"/>
-    </row>
-    <row r="26" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="20"/>
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="35"/>
-      <c r="H26" s="30"/>
-    </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="20"/>
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="44"/>
-    </row>
-    <row r="28" spans="1:8" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="20"/>
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="29"/>
-    </row>
-    <row r="29" spans="1:8" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="20"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="32"/>
-      <c r="H29" s="29"/>
-    </row>
-    <row r="30" spans="1:8" ht="73.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="20"/>
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="29"/>
-    </row>
-    <row r="31" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="20"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="30"/>
-    </row>
-    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="20"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="35"/>
-      <c r="H32" s="44"/>
-    </row>
-    <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="18"/>
-      <c r="B33" s="39"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="47"/>
-      <c r="H33" s="23"/>
-    </row>
-    <row r="34" spans="1:8" ht="1.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="28"/>
-      <c r="B34" s="50"/>
-      <c r="C34" s="50"/>
-      <c r="D34" s="50"/>
-      <c r="E34" s="50"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="26"/>
-    </row>
-    <row r="35" spans="1:8" ht="8.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="28"/>
-      <c r="B35" s="50"/>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="47"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="44"/>
-    </row>
-    <row r="36" spans="1:8" ht="4.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="4"/>
-      <c r="H36" s="5"/>
-    </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="4"/>
-      <c r="H37" s="5"/>
-    </row>
-    <row r="38" spans="1:8" ht="9.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="4"/>
-      <c r="H38" s="5"/>
-    </row>
-    <row r="39" spans="1:8" ht="7.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="4"/>
-      <c r="H39" s="5"/>
-    </row>
-    <row r="40" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="4"/>
-      <c r="E40" s="43"/>
-      <c r="F40" s="36"/>
-      <c r="G40" s="36"/>
-      <c r="H40" s="45"/>
-    </row>
-    <row r="41" spans="1:8" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="4"/>
-      <c r="H41" s="46"/>
-    </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="18"/>
-      <c r="B42" s="39"/>
-      <c r="C42" s="39"/>
-      <c r="D42" s="39"/>
-      <c r="H42" s="46"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" s="4"/>
-      <c r="E43" s="2" t="s">
+    <row r="24" spans="1:8" ht="1.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="28"/>
+      <c r="B24" s="44"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="26"/>
+    </row>
+    <row r="25" spans="1:8" ht="8.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="28"/>
+      <c r="B25" s="44"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="38"/>
+    </row>
+    <row r="26" spans="1:8" ht="4.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="4"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="4"/>
+      <c r="H27" s="5"/>
+    </row>
+    <row r="28" spans="1:8" ht="9.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="4"/>
+      <c r="H28" s="5"/>
+    </row>
+    <row r="29" spans="1:8" ht="7.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="4"/>
+      <c r="H29" s="5"/>
+    </row>
+    <row r="30" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="4"/>
+      <c r="E30" s="37"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="39"/>
+    </row>
+    <row r="31" spans="1:8" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="4"/>
+      <c r="H31" s="40"/>
+    </row>
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="18"/>
+      <c r="B32" s="33"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="H32" s="40"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="4"/>
+      <c r="E33" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-      <c r="H43" s="3"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="4"/>
-      <c r="E44" t="s">
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="3"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34" s="4"/>
+      <c r="E34" t="s">
         <v>15</v>
       </c>
-      <c r="H44" s="5"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="6"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="7" t="s">
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35" s="6"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F45" s="7"/>
-      <c r="G45" s="7"/>
-      <c r="H45" s="8"/>
-    </row>
-    <row r="47" spans="1:8" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="8"/>
+    </row>
+    <row r="37" spans="1:8" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
         <v>17</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F37" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="25.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:8" ht="25.2" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:H1"/>

</xml_diff>